<commit_message>
Diversify synthetic care-package labels across five service types
Replace the uniform "Supported Living" with a realistic, service-weighted mix
of adult social care service types — Supported Living, Residential Care,
Community Outreach, Complex Support, Day Support — in both:
- seed.ts (app demo data): PACKAGE_MIX weighted per service
- CQI_Synthetic_Quality_Sample_Data.xlsx Clients sheet (all 60 rows), also
  clearing leftover "Respite"/"Live-in" values

All data remains synthetic: no real provider names, service-user names, staff
performance or addresses.

Verified: grep "Aldanat"/"Domiciliary" → none; npm run lint → clean;
npm run build → passes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CQI_Synthetic_Quality_Sample_Data.xlsx
+++ b/CQI_Synthetic_Quality_Sample_Data.xlsx
@@ -1700,7 +1700,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Complex Support</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Live-in</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Complex Support</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Live-in</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Live-in</t>
+          <t>Complex Support</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Live-in</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Complex Support</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Live-in</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Live-in</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Complex Support</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Complex Support</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Live-in</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Complex Support</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Respite</t>
+          <t>Community Outreach</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Residential Care</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Live-in</t>
+          <t>Day Support</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">

</xml_diff>